<commit_message>
chore: sincroniza acervo completo e resultados históricos do ORCA-AI
Inclui orçamentos, documentos de governança, arquivo histórico e todas as execuções de ML preservadas. Concilia o conteúdo com o OneDrive e registra as verificações e a ressalva editorial dos despachos.
</commit_message>
<xml_diff>
--- a/OrcaAI/projetos/Item 01 - teto_elevadores/Composicao de BDI - teto dos elevadores.xlsx
+++ b/OrcaAI/projetos/Item 01 - teto_elevadores/Composicao de BDI - teto dos elevadores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/044143bd5bee1bfc/04 - Meus Documentos/GitHub/Orcamento_de_Obra/Item 01 - teto_elevadores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A0FD7FC-7463-4E09-9A53-A199F24A3A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{3A0FD7FC-7463-4E09-9A53-A199F24A3A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADE0CBDE-1247-4F4F-A283-D7D3D9DB8E0D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1362,8 +1362,8 @@
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="A3:L3"/>
   </mergeCells>
-  <pageMargins left="0.5" right="0.5" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="77" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L &amp;C &amp;R</oddHeader>
     <oddFooter>&amp;L &amp;C &amp;R</oddFooter>
@@ -1371,6 +1371,6 @@
   <ignoredErrors>
     <ignoredError sqref="F2 A5:L30" numberStoredAsText="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>